<commit_message>
qa: add execution status dropdown to Sprint 3 trace
</commit_message>
<xml_diff>
--- a/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
+++ b/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R81e21a48109e4ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R7eef7ab114d94cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R36c8daa800444ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="Rea33eda1032442b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1365,6 +1365,11 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G6:G49">
+      <x:formula1>"Not Executed,In Progress,Pending,Passed,Failed,Blocked,Skipped,Retest"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
qa: map Sprint 3 QR Rewards trace to Phase 2 cases
</commit_message>
<xml_diff>
--- a/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
+++ b/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R36c8daa800444ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="Rea33eda1032442b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R490cede8f29149ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R750c44def0284d59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,8 +42,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,6 +59,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1E3A5F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF274E72"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF1F8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -68,7 +84,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -82,6 +98,19 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -296,6 +325,9 @@
     <x:col min="5" max="5" width="53" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -329,7 +361,7 @@
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
+    <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="5" t="str">
         <x:v>TC ID</x:v>
       </x:c>
@@ -351,8 +383,17 @@
       <x:c r="G5" s="5" t="str">
         <x:v>Execution</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="H5" s="12" t="str">
+        <x:v>Phase 2 TC ID liên kết</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>Mức độ đối chiếu</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>Phần còn thiếu / điều kiện chốt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>QR-001</x:v>
       </x:c>
@@ -374,8 +415,17 @@
       <x:c r="G6" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="H6" s="7" t="str">
+        <x:v>P2-QR-002; P2-QR-015</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="str">
+        <x:v>Zero-login và mốc ≤30 giây có hai case P2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>QR-002</x:v>
       </x:c>
@@ -397,8 +447,17 @@
       <x:c r="G7" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="H7" s="7" t="str">
+        <x:v>P2-QR-002; P2-RWD-001</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J7" s="7" t="str">
+        <x:v>Chưa có assertion riêng: bỏ qua số điện thoại vẫn đặt món được.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="7" t="str">
         <x:v>QR-003</x:v>
       </x:c>
@@ -420,8 +479,17 @@
       <x:c r="G8" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="H8" s="7" t="str">
+        <x:v>P2-QR-001; P2-QR-003</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J8" s="7" t="str">
+        <x:v>Token, table và session phải cùng fixture.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="7" t="str">
         <x:v>QR-004</x:v>
       </x:c>
@@ -443,8 +511,17 @@
       <x:c r="G9" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="H9" s="7" t="str">
+        <x:v>P2-QR-007</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J9" s="7" t="str">
+        <x:v>Chờ BE định nghĩa TTL, revoke và error response.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>QR-005</x:v>
       </x:c>
@@ -466,8 +543,17 @@
       <x:c r="G10" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="H10" s="7" t="str">
+        <x:v>P2-QR-001; P2-QR-008</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J10" s="7" t="str">
+        <x:v>Chưa có tình huống tấm QR đặt nhầm bàn và cách khách xác nhận bàn.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="7" t="str">
         <x:v>QR-006</x:v>
       </x:c>
@@ -489,8 +575,17 @@
       <x:c r="G11" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="H11" s="7" t="str">
+        <x:v>P2-QR-002</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J11" s="7" t="str">
+        <x:v>Món unavailable không chọn được.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>QR-007</x:v>
       </x:c>
@@ -512,8 +607,17 @@
       <x:c r="G12" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="H12" s="7" t="str">
+        <x:v>P2-QR-002</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J12" s="7" t="str">
+        <x:v>P2 chỉ kiểm menu; thiếu race item hết hàng sau khi mở cart, trước checkout.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="7" t="str">
         <x:v>QR-008</x:v>
       </x:c>
@@ -535,8 +639,17 @@
       <x:c r="G13" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="H13" s="7" t="str">
+        <x:v>P2-QR-006</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J13" s="7" t="str">
+        <x:v>Hai request ID và hai giỏ độc lập cùng session.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="7" t="str">
         <x:v>QR-009</x:v>
       </x:c>
@@ -558,8 +671,17 @@
       <x:c r="G14" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="H14" s="7" t="str">
+        <x:v>P2-QR-004</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J14" s="7" t="str">
+        <x:v>POS + QR cùng active session.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="7" t="str">
         <x:v>QR-010</x:v>
       </x:c>
@@ -581,8 +703,17 @@
       <x:c r="G15" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="H15" s="7" t="str">
+        <x:v>P2-QR-005</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J15" s="7" t="str">
+        <x:v>BRD gọi request_id; chờ BE xác nhận key/payload replay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="7" t="str">
         <x:v>QR-011</x:v>
       </x:c>
@@ -604,8 +735,17 @@
       <x:c r="G16" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="H16" s="7" t="str">
+        <x:v>P2-QR-005</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J16" s="7" t="str">
+        <x:v>Thiếu assertion cùng request_id khác body: conflict và không mutation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="7" t="str">
         <x:v>QR-012</x:v>
       </x:c>
@@ -627,8 +767,17 @@
       <x:c r="G17" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="H17" s="7" t="str">
+        <x:v>P2-QR-014</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J17" s="7" t="str">
+        <x:v>Retry sau mất response không tạo thêm order/ticket.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="7" t="str">
         <x:v>QR-013</x:v>
       </x:c>
@@ -650,8 +799,17 @@
       <x:c r="G18" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="H18" s="7" t="str">
+        <x:v>P2-QR-009</x:v>
+      </x:c>
+      <x:c r="I18" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J18" s="7" t="str">
+        <x:v>Không sửa order QR sau submit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="7" t="str">
         <x:v>QR-014</x:v>
       </x:c>
@@ -673,8 +831,17 @@
       <x:c r="G19" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="H19" s="7" t="str">
+        <x:v>P2-QR-013</x:v>
+      </x:c>
+      <x:c r="I19" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J19" s="7" t="str">
+        <x:v>Billing khóa gửi QR đúng session.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="7" t="str">
         <x:v>QR-015</x:v>
       </x:c>
@@ -696,8 +863,17 @@
       <x:c r="G20" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="H20" s="7" t="str">
+        <x:v>P2-QR-003; P2-QR-011</x:v>
+      </x:c>
+      <x:c r="I20" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J20" s="7" t="str">
+        <x:v>P2 có SENT và modifier routing; cần case routing QR không modifier theo station.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="7" t="str">
         <x:v>QR-016</x:v>
       </x:c>
@@ -719,8 +895,17 @@
       <x:c r="G21" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="H21" s="7" t="str">
+        <x:v>P2-QR-011; P2-QR-012</x:v>
+      </x:c>
+      <x:c r="I21" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J21" s="7" t="str">
+        <x:v>Modifier có; ghi chú món QR chưa có assertion riêng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="7" t="str">
         <x:v>QR-017</x:v>
       </x:c>
@@ -742,8 +927,15 @@
       <x:c r="G22" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="H22" s="7" t="str"/>
+      <x:c r="I22" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J22" s="7" t="str">
+        <x:v>Thêm case UI QR realtime/status và resync theo contract FE/BE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="7" t="str">
         <x:v>QR-018</x:v>
       </x:c>
@@ -765,8 +957,17 @@
       <x:c r="G23" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="H23" s="7" t="str">
+        <x:v>P2-QR-007</x:v>
+      </x:c>
+      <x:c r="I23" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J23" s="7" t="str">
+        <x:v>P2 chỉ kiểm token; thiếu idle/cart retention và expiry trong lúc có giỏ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="7" t="str">
         <x:v>QR-019</x:v>
       </x:c>
@@ -788,8 +989,17 @@
       <x:c r="G24" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="H24" s="7" t="str">
+        <x:v>P2-QR-007; P2-QR-008</x:v>
+      </x:c>
+      <x:c r="I24" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J24" s="7" t="str">
+        <x:v>Token tamper và cross-table read/write.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="7" t="str">
         <x:v>QR-020</x:v>
       </x:c>
@@ -811,8 +1021,17 @@
       <x:c r="G25" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="H25" s="7" t="str">
+        <x:v>P2-QR-004; P2-AUD-005</x:v>
+      </x:c>
+      <x:c r="I25" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J25" s="7" t="str">
+        <x:v>Bill/session có; thiếu assertion source QR/POS và audit merge trong cùng case.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="7" t="str">
         <x:v>QR-021</x:v>
       </x:c>
@@ -834,8 +1053,17 @@
       <x:c r="G26" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="H26" s="7" t="str">
+        <x:v>P2-TBL-004</x:v>
+      </x:c>
+      <x:c r="I26" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J26" s="7" t="str">
+        <x:v>Transfer giữ QR association; phụ thuộc advanced table.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="7" t="str">
         <x:v>QR-022</x:v>
       </x:c>
@@ -857,8 +1085,15 @@
       <x:c r="G27" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="H27" s="7" t="str"/>
+      <x:c r="I27" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J27" s="7" t="str">
+        <x:v>MAIN sau course fired cần PO chốt policy trước khi tạo case.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="7" t="str">
         <x:v>QR-023</x:v>
       </x:c>
@@ -880,8 +1115,17 @@
       <x:c r="G28" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="H28" s="7" t="str">
+        <x:v>P2-QR-014</x:v>
+      </x:c>
+      <x:c r="I28" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J28" s="7" t="str">
+        <x:v>P2 retry khi QR mất mạng; POS offline nhưng QR online là nhánh khác.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="7" t="str">
         <x:v>QR-024</x:v>
       </x:c>
@@ -903,8 +1147,15 @@
       <x:c r="G29" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30" ht="30" customHeight="1">
+      <x:c r="H29" s="7" t="str"/>
+      <x:c r="I29" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J29" s="7" t="str">
+        <x:v>Bếp quá tải/capacity fixture chưa có case P2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="7" t="str">
         <x:v>RW-001</x:v>
       </x:c>
@@ -926,8 +1177,17 @@
       <x:c r="G30" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="H30" s="7" t="str">
+        <x:v>P2-RWD-001</x:v>
+      </x:c>
+      <x:c r="I30" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J30" s="7" t="str">
+        <x:v>Nhận diện theo số điện thoại; chờ PII policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="7" t="str">
         <x:v>RW-002</x:v>
       </x:c>
@@ -949,8 +1209,15 @@
       <x:c r="G31" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="H31" s="7" t="str"/>
+      <x:c r="I31" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J31" s="7" t="str">
+        <x:v>Mã thành viên là phương thức nhận diện riêng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="7" t="str">
         <x:v>RW-003</x:v>
       </x:c>
@@ -972,8 +1239,17 @@
       <x:c r="G32" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="H32" s="7" t="str">
+        <x:v>P2-QR-002; P2-RWD-001</x:v>
+      </x:c>
+      <x:c r="I32" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J32" s="7" t="str">
+        <x:v>Chưa có assertion khách bỏ qua Rewards nhưng vẫn thanh toán bình thường.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="7" t="str">
         <x:v>RW-004</x:v>
       </x:c>
@@ -995,8 +1271,17 @@
       <x:c r="G33" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="30" customHeight="1">
+      <x:c r="H33" s="7" t="str">
+        <x:v>P2-RWD-003; P2-RWD-004</x:v>
+      </x:c>
+      <x:c r="I33" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J33" s="7" t="str">
+        <x:v>Tra reward và eligibility theo rule PO.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="7" t="str">
         <x:v>RW-005</x:v>
       </x:c>
@@ -1018,8 +1303,17 @@
       <x:c r="G34" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="H34" s="7" t="str">
+        <x:v>P2-RWD-005</x:v>
+      </x:c>
+      <x:c r="I34" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J34" s="7" t="str">
+        <x:v>Áp reward hợp lệ vào bill chưa trả.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="7" t="str">
         <x:v>RW-006</x:v>
       </x:c>
@@ -1041,8 +1335,17 @@
       <x:c r="G35" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="H35" s="7" t="str">
+        <x:v>P2-RWD-004</x:v>
+      </x:c>
+      <x:c r="I35" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J35" s="7" t="str">
+        <x:v>P2 eligibility chung; cần riêng expired/used/insufficient points.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="7" t="str">
         <x:v>RW-007</x:v>
       </x:c>
@@ -1064,8 +1367,15 @@
       <x:c r="G36" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37" ht="30" customHeight="1">
+      <x:c r="H36" s="7" t="str"/>
+      <x:c r="I36" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J36" s="7" t="str">
+        <x:v>Thiếu conflict stacking giữa các reward/promotion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="7" t="str">
         <x:v>RW-008</x:v>
       </x:c>
@@ -1087,8 +1397,15 @@
       <x:c r="G37" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="H37" s="7" t="str"/>
+      <x:c r="I37" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J37" s="7" t="str">
+        <x:v>Thiếu giới hạn khuyến mãi theo cấu hình/rule version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="7" t="str">
         <x:v>RW-009</x:v>
       </x:c>
@@ -1110,8 +1427,15 @@
       <x:c r="G38" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="H38" s="7" t="str"/>
+      <x:c r="I38" s="7" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="J38" s="7" t="str">
+        <x:v>Thiếu Supervisor override và audit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="7" t="str">
         <x:v>RW-010</x:v>
       </x:c>
@@ -1133,8 +1457,17 @@
       <x:c r="G39" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="H39" s="7" t="str">
+        <x:v>P2-RWD-006</x:v>
+      </x:c>
+      <x:c r="I39" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J39" s="7" t="str">
+        <x:v>P2 double-use; retry cùng request key cần assertion ledger một lần.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="7" t="str">
         <x:v>RW-011</x:v>
       </x:c>
@@ -1156,8 +1489,17 @@
       <x:c r="G40" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="H40" s="7" t="str">
+        <x:v>P2-RWD-006</x:v>
+      </x:c>
+      <x:c r="I40" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J40" s="7" t="str">
+        <x:v>Concurrent redeem trên hai bill; balance không âm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="7" t="str">
         <x:v>RW-012</x:v>
       </x:c>
@@ -1179,8 +1521,17 @@
       <x:c r="G41" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="H41" s="7" t="str">
+        <x:v>P2-RWD-009</x:v>
+      </x:c>
+      <x:c r="I41" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J41" s="7" t="str">
+        <x:v>Payment failure có; CRM unavailable nhưng payment fallback cần case riêng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" s="7" t="str">
         <x:v>RW-013</x:v>
       </x:c>
@@ -1202,8 +1553,17 @@
       <x:c r="G42" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="H42" s="7" t="str">
+        <x:v>P2-RWD-005</x:v>
+      </x:c>
+      <x:c r="I42" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J42" s="7" t="str">
+        <x:v>≤30 giây tạm theo mục tiêu; PO cần chốt với risk note ≤10 giây.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="7" t="str">
         <x:v>RW-014</x:v>
       </x:c>
@@ -1225,8 +1585,17 @@
       <x:c r="G43" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="H43" s="7" t="str">
+        <x:v>P2-RWD-007</x:v>
+      </x:c>
+      <x:c r="I43" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J43" s="7" t="str">
+        <x:v>Gỡ reward trước pay và hoàn nguyên ledger.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="7" t="str">
         <x:v>RW-015</x:v>
       </x:c>
@@ -1248,8 +1617,17 @@
       <x:c r="G44" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="H44" s="7" t="str">
+        <x:v>P2-RWD-010</x:v>
+      </x:c>
+      <x:c r="I44" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J44" s="7" t="str">
+        <x:v>Không lộ PII/points cross-customer/outlet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" s="7" t="str">
         <x:v>RW-016</x:v>
       </x:c>
@@ -1271,8 +1649,17 @@
       <x:c r="G45" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="46" ht="30" customHeight="1">
+      <x:c r="H45" s="7" t="str">
+        <x:v>P2-RWD-009</x:v>
+      </x:c>
+      <x:c r="I45" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J45" s="7" t="str">
+        <x:v>P2 payment failed; refund/hủy sau pay và reversal thiếu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" s="7" t="str">
         <x:v>RW-017</x:v>
       </x:c>
@@ -1294,8 +1681,17 @@
       <x:c r="G46" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="H46" s="7" t="str">
+        <x:v>P2-RWD-004</x:v>
+      </x:c>
+      <x:c r="I46" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J46" s="7" t="str">
+        <x:v>Eligibility lần đầu có; thay bill rồi tính lại chưa có.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" s="7" t="str">
         <x:v>RW-018</x:v>
       </x:c>
@@ -1317,8 +1713,17 @@
       <x:c r="G47" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48" ht="30" customHeight="1">
+      <x:c r="H47" s="7" t="str">
+        <x:v>P2-RWD-011</x:v>
+      </x:c>
+      <x:c r="I47" s="7" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="J47" s="7" t="str">
+        <x:v>Earn đúng một lần sau PAID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" s="7" t="str">
         <x:v>RW-019</x:v>
       </x:c>
@@ -1340,8 +1745,17 @@
       <x:c r="G48" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49" ht="30" customHeight="1">
+      <x:c r="H48" s="7" t="str">
+        <x:v>P2-RWD-003; P2-RWD-011</x:v>
+      </x:c>
+      <x:c r="I48" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J48" s="7" t="str">
+        <x:v>Earn/balance có; thiếu ledger redemption/reversal đầy đủ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" s="7" t="str">
         <x:v>RW-020</x:v>
       </x:c>
@@ -1363,11 +1777,97 @@
       <x:c r="G49" s="7" t="str">
         <x:v>Not Executed</x:v>
       </x:c>
+      <x:c r="H49" s="7" t="str">
+        <x:v>P2-RWD-005</x:v>
+      </x:c>
+      <x:c r="I49" s="7" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="J49" s="7" t="str">
+        <x:v>P2 apply reward có; thiếu giả mạo discount từ client.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="14" t="str">
+        <x:v>Đối chiếu 44 case Sprint 3 với bộ 71 Pha 2</x:v>
+      </x:c>
+      <x:c r="B51" s="14"/>
+      <x:c r="C51" s="14"/>
+      <x:c r="D51" s="14"/>
+      <x:c r="E51" s="14"/>
+      <x:c r="F51" s="14"/>
+      <x:c r="G51" s="14"/>
+      <x:c r="H51" s="14"/>
+      <x:c r="I51" s="14"/>
+      <x:c r="J51" s="14"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>Khớp</x:v>
+      </x:c>
+      <x:c r="B52" t="n">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+      <x:c r="B53" t="n">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>Chưa có P2 tương ứng</x:v>
+      </x:c>
+      <x:c r="B54" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="38" customHeight="1">
+      <x:c r="A55" t="str">
+        <x:v>P2 QR/RWD chưa có Sprint 3 ID trực tiếp</x:v>
+      </x:c>
+      <x:c r="B55" s="15" t="str">
+        <x:v>P2-QR-010; P2-RWD-002; P2-RWD-008</x:v>
+      </x:c>
+      <x:c r="C55" s="15"/>
+      <x:c r="D55" s="15"/>
+      <x:c r="E55" s="15"/>
+      <x:c r="F55" s="15"/>
+      <x:c r="G55" s="15"/>
+      <x:c r="H55" s="15"/>
+      <x:c r="I55" s="15"/>
+      <x:c r="J55" s="15"/>
+    </x:row>
+    <x:row r="56" ht="38" customHeight="1">
+      <x:c r="A56" t="str">
+        <x:v>Lưu ý</x:v>
+      </x:c>
+      <x:c r="B56" s="15" t="str">
+        <x:v>Đối chiếu thiết kế, không cộng 44 và 71 thành số testcase thực thi. Rewards policy và API/fixture còn chờ PO/BE/CRM.</x:v>
+      </x:c>
+      <x:c r="C56" s="15"/>
+      <x:c r="D56" s="15"/>
+      <x:c r="E56" s="15"/>
+      <x:c r="F56" s="15"/>
+      <x:c r="G56" s="15"/>
+      <x:c r="H56" s="15"/>
+      <x:c r="I56" s="15"/>
+      <x:c r="J56" s="15"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:mergeCells>
+    <x:mergeCell ref="B55:J55"/>
+    <x:mergeCell ref="B56:J56"/>
+  </x:mergeCells>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G6:G49">
       <x:formula1>"Not Executed,In Progress,Pending,Passed,Failed,Blocked,Skipped,Retest"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I6:I49">
+      <x:formula1>"Khớp,Một phần,Chưa có P2 tương ứng"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
qa: triage Sprint 3 QR Rewards trace against BRD
</commit_message>
<xml_diff>
--- a/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
+++ b/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R490cede8f29149ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R750c44def0284d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R108336a74ceb42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R8290e56d2b724076"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +71,11 @@
         <x:fgColor rgb="FFEAF1F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF274E72"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -84,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -112,6 +117,14 @@
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -328,6 +341,8 @@
     <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -392,8 +407,14 @@
       <x:c r="J5" s="12" t="str">
         <x:v>Phần còn thiếu / điều kiện chốt</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="K5" s="19" t="str">
+        <x:v>Xử lý QA 27/10</x:v>
+      </x:c>
+      <x:c r="L5" s="19" t="str">
+        <x:v>Assertion / quyết định còn thiếu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="50" customHeight="1">
       <x:c r="A6" s="7" t="str">
         <x:v>QR-001</x:v>
       </x:c>
@@ -424,8 +445,10 @@
       <x:c r="J6" s="7" t="str">
         <x:v>Zero-login và mốc ≤30 giây có hai case P2.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="K6" s="7" t="str"/>
+      <x:c r="L6" s="7" t="str"/>
+    </x:row>
+    <x:row r="7" ht="50" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>QR-002</x:v>
       </x:c>
@@ -456,8 +479,14 @@
       <x:c r="J7" s="7" t="str">
         <x:v>Chưa có assertion riêng: bỏ qua số điện thoại vẫn đặt món được.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="K7" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L7" s="7" t="str">
+        <x:v>Không nhập số điện thoại vẫn xem menu và gửi order. BR-QR-003; không ràng buộc Rewards.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="50" customHeight="1">
       <x:c r="A8" s="7" t="str">
         <x:v>QR-003</x:v>
       </x:c>
@@ -488,8 +517,10 @@
       <x:c r="J8" s="7" t="str">
         <x:v>Token, table và session phải cùng fixture.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="K8" s="7" t="str"/>
+      <x:c r="L8" s="7" t="str"/>
+    </x:row>
+    <x:row r="9" ht="50" customHeight="1">
       <x:c r="A9" s="7" t="str">
         <x:v>QR-004</x:v>
       </x:c>
@@ -520,8 +551,10 @@
       <x:c r="J9" s="7" t="str">
         <x:v>Chờ BE định nghĩa TTL, revoke và error response.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="K9" s="7" t="str"/>
+      <x:c r="L9" s="7" t="str"/>
+    </x:row>
+    <x:row r="10" ht="50" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>QR-005</x:v>
       </x:c>
@@ -550,10 +583,16 @@
         <x:v>Một phần</x:v>
       </x:c>
       <x:c r="J10" s="7" t="str">
-        <x:v>Chưa có tình huống tấm QR đặt nhầm bàn và cách khách xác nhận bàn.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="48" customHeight="1">
+        <x:v>BRD QR Edge Cases: QR đặt nhầm bàn không tự bị chặn; order theo bàn của QR, nhân viên xử lý. P2 chưa có ca kiểm thực địa.</x:v>
+      </x:c>
+      <x:c r="K10" s="7" t="str">
+        <x:v>Sửa expected từ BRD</x:v>
+      </x:c>
+      <x:c r="L10" s="7" t="str">
+        <x:v>QR đặt nhầm bàn dẫn order theo QR đã quét; nhân viên xử lý. BRD QR Edge Cases; không kỳ vọng chặn tự động.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
       <x:c r="A11" s="7" t="str">
         <x:v>QR-006</x:v>
       </x:c>
@@ -584,8 +623,10 @@
       <x:c r="J11" s="7" t="str">
         <x:v>Món unavailable không chọn được.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="48" customHeight="1">
+      <x:c r="K11" s="7" t="str"/>
+      <x:c r="L11" s="7" t="str"/>
+    </x:row>
+    <x:row r="12" ht="50" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>QR-007</x:v>
       </x:c>
@@ -614,10 +655,16 @@
         <x:v>Một phần</x:v>
       </x:c>
       <x:c r="J12" s="7" t="str">
-        <x:v>P2 chỉ kiểm menu; thiếu race item hết hàng sau khi mở cart, trước checkout.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+        <x:v>BRD QR Edge Cases: hết hàng lúc checkout phải chặn submit và hiển thị lỗi món; thiếu race assertion trong P2.</x:v>
+      </x:c>
+      <x:c r="K12" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L12" s="7" t="str">
+        <x:v>Món hết hàng ngay checkout: chặn submit, hiện lỗi món; không tạo order/ticket. BRD QR Edge Cases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
       <x:c r="A13" s="7" t="str">
         <x:v>QR-008</x:v>
       </x:c>
@@ -648,8 +695,10 @@
       <x:c r="J13" s="7" t="str">
         <x:v>Hai request ID và hai giỏ độc lập cùng session.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="K13" s="7" t="str"/>
+      <x:c r="L13" s="7" t="str"/>
+    </x:row>
+    <x:row r="14" ht="50" customHeight="1">
       <x:c r="A14" s="7" t="str">
         <x:v>QR-009</x:v>
       </x:c>
@@ -680,8 +729,10 @@
       <x:c r="J14" s="7" t="str">
         <x:v>POS + QR cùng active session.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="K14" s="7" t="str"/>
+      <x:c r="L14" s="7" t="str"/>
+    </x:row>
+    <x:row r="15" ht="50" customHeight="1">
       <x:c r="A15" s="7" t="str">
         <x:v>QR-010</x:v>
       </x:c>
@@ -712,8 +763,10 @@
       <x:c r="J15" s="7" t="str">
         <x:v>BRD gọi request_id; chờ BE xác nhận key/payload replay.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="K15" s="7" t="str"/>
+      <x:c r="L15" s="7" t="str"/>
+    </x:row>
+    <x:row r="16" ht="50" customHeight="1">
       <x:c r="A16" s="7" t="str">
         <x:v>QR-011</x:v>
       </x:c>
@@ -744,8 +797,14 @@
       <x:c r="J16" s="7" t="str">
         <x:v>Thiếu assertion cùng request_id khác body: conflict và không mutation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="48" customHeight="1">
+      <x:c r="K16" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L16" s="7" t="str">
+        <x:v>Cùng request_id, khác body: không tạo thêm order/ticket; mã HTTP và replay/conflict chờ BE. BR-QR-005.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="50" customHeight="1">
       <x:c r="A17" s="7" t="str">
         <x:v>QR-012</x:v>
       </x:c>
@@ -776,8 +835,10 @@
       <x:c r="J17" s="7" t="str">
         <x:v>Retry sau mất response không tạo thêm order/ticket.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="K17" s="7" t="str"/>
+      <x:c r="L17" s="7" t="str"/>
+    </x:row>
+    <x:row r="18" ht="50" customHeight="1">
       <x:c r="A18" s="7" t="str">
         <x:v>QR-013</x:v>
       </x:c>
@@ -808,8 +869,10 @@
       <x:c r="J18" s="7" t="str">
         <x:v>Không sửa order QR sau submit.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="48" customHeight="1">
+      <x:c r="K18" s="7" t="str"/>
+      <x:c r="L18" s="7" t="str"/>
+    </x:row>
+    <x:row r="19" ht="50" customHeight="1">
       <x:c r="A19" s="7" t="str">
         <x:v>QR-014</x:v>
       </x:c>
@@ -840,8 +903,10 @@
       <x:c r="J19" s="7" t="str">
         <x:v>Billing khóa gửi QR đúng session.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="K19" s="7" t="str"/>
+      <x:c r="L19" s="7" t="str"/>
+    </x:row>
+    <x:row r="20" ht="50" customHeight="1">
       <x:c r="A20" s="7" t="str">
         <x:v>QR-015</x:v>
       </x:c>
@@ -872,8 +937,14 @@
       <x:c r="J20" s="7" t="str">
         <x:v>P2 có SENT và modifier routing; cần case routing QR không modifier theo station.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="K20" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L20" s="7" t="str">
+        <x:v>Món QR chỉ tới Kitchen khi SENT và station_id đúng; fixture có hai trạm, không giả định đủ sáu trạm. BR-QR-006.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="50" customHeight="1">
       <x:c r="A21" s="7" t="str">
         <x:v>QR-016</x:v>
       </x:c>
@@ -904,8 +975,14 @@
       <x:c r="J21" s="7" t="str">
         <x:v>Modifier có; ghi chú món QR chưa có assertion riêng.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="48" customHeight="1">
+      <x:c r="K21" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L21" s="7" t="str">
+        <x:v>Kiểm ghi chú lưu trên item và hiển thị cho bếp; Modifier/routing phụ thuộc schema BE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="50" customHeight="1">
       <x:c r="A22" s="7" t="str">
         <x:v>QR-017</x:v>
       </x:c>
@@ -934,8 +1011,14 @@
       <x:c r="J22" s="7" t="str">
         <x:v>Thêm case UI QR realtime/status và resync theo contract FE/BE.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="48" customHeight="1">
+      <x:c r="K22" s="7" t="str">
+        <x:v>Đề xuất testcase P2</x:v>
+      </x:c>
+      <x:c r="L22" s="7" t="str">
+        <x:v>Thêm QR UI trạng thái món và đồng bộ sau reconnect; cần FE route/event và BE read/status contract.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="50" customHeight="1">
       <x:c r="A23" s="7" t="str">
         <x:v>QR-018</x:v>
       </x:c>
@@ -966,8 +1049,14 @@
       <x:c r="J23" s="7" t="str">
         <x:v>P2 chỉ kiểm token; thiếu idle/cart retention và expiry trong lúc có giỏ.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="48" customHeight="1">
+      <x:c r="K23" s="7" t="str">
+        <x:v>Chờ PO chốt thời hạn</x:v>
+      </x:c>
+      <x:c r="L23" s="7" t="str">
+        <x:v>BRD ghi giữ cart X phút, chưa định X và quan hệ token expiry; chuẩn bị các mốc trước/sau X.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="50" customHeight="1">
       <x:c r="A24" s="7" t="str">
         <x:v>QR-019</x:v>
       </x:c>
@@ -998,8 +1087,10 @@
       <x:c r="J24" s="7" t="str">
         <x:v>Token tamper và cross-table read/write.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="48" customHeight="1">
+      <x:c r="K24" s="7" t="str"/>
+      <x:c r="L24" s="7" t="str"/>
+    </x:row>
+    <x:row r="25" ht="50" customHeight="1">
       <x:c r="A25" s="7" t="str">
         <x:v>QR-020</x:v>
       </x:c>
@@ -1030,8 +1121,14 @@
       <x:c r="J25" s="7" t="str">
         <x:v>Bill/session có; thiếu assertion source QR/POS và audit merge trong cùng case.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="48" customHeight="1">
+      <x:c r="K25" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L25" s="7" t="str">
+        <x:v>QR+POS: bill gộp item chưa trả, source từng item còn truy vết, audit được giữ. BR-OM-MRG-004/006/008.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="50" customHeight="1">
       <x:c r="A26" s="7" t="str">
         <x:v>QR-021</x:v>
       </x:c>
@@ -1062,8 +1159,10 @@
       <x:c r="J26" s="7" t="str">
         <x:v>Transfer giữ QR association; phụ thuộc advanced table.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="48" customHeight="1">
+      <x:c r="K26" s="7" t="str"/>
+      <x:c r="L26" s="7" t="str"/>
+    </x:row>
+    <x:row r="27" ht="50" customHeight="1">
       <x:c r="A27" s="7" t="str">
         <x:v>QR-022</x:v>
       </x:c>
@@ -1090,10 +1189,16 @@
         <x:v>Chưa có P2 tương ứng</x:v>
       </x:c>
       <x:c r="J27" s="7" t="str">
-        <x:v>MAIN sau course fired cần PO chốt policy trước khi tạo case.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="48" customHeight="1">
+        <x:v>BRD Course Firing Edge Cases: MAIN thêm sau khi fired vẫn CREATED, Waiter fire riêng; chưa có testcase P2 trực tiếp.</x:v>
+      </x:c>
+      <x:c r="K27" s="7" t="str">
+        <x:v>Đề xuất testcase P2</x:v>
+      </x:c>
+      <x:c r="L27" s="7" t="str">
+        <x:v>BRD Course Firing Edge Cases: MAIN QR thêm sau khi đã fired vẫn CREATED; Waiter phải fire riêng; không tạo ticket trước fire.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="50" customHeight="1">
       <x:c r="A28" s="7" t="str">
         <x:v>QR-023</x:v>
       </x:c>
@@ -1122,10 +1227,16 @@
         <x:v>Một phần</x:v>
       </x:c>
       <x:c r="J28" s="7" t="str">
-        <x:v>P2 retry khi QR mất mạng; POS offline nhưng QR online là nhánh khác.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="48" customHeight="1">
+        <x:v>BRD Merge/Offline Edge Cases: POS offline nhưng QR online, queue/sync khi POS nối lại; khác retry khi QR mất mạng.</x:v>
+      </x:c>
+      <x:c r="K28" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L28" s="7" t="str">
+        <x:v>POS offline, QR online: queue/sync QR khi POS nối lại; không mất hoặc nhân đôi order. BRD Merge/Offline Edge Cases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="50" customHeight="1">
       <x:c r="A29" s="7" t="str">
         <x:v>QR-024</x:v>
       </x:c>
@@ -1152,10 +1263,16 @@
         <x:v>Chưa có P2 tương ứng</x:v>
       </x:c>
       <x:c r="J29" s="7" t="str">
-        <x:v>Bếp quá tải/capacity fixture chưa có case P2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="48" customHeight="1">
+        <x:v>BRD QR Edge Cases: bếp quá tải vẫn nhận order, SLA theo dõi trễ; P2 thiếu case và fixture tải.</x:v>
+      </x:c>
+      <x:c r="K29" s="7" t="str">
+        <x:v>Đề xuất testcase P2</x:v>
+      </x:c>
+      <x:c r="L29" s="7" t="str">
+        <x:v>BRD QR Edge Cases: vẫn nhận order khi bếp quá tải, SLA theo dõi trễ; cần fixture tải có kiểm soát.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="50" customHeight="1">
       <x:c r="A30" s="7" t="str">
         <x:v>RW-001</x:v>
       </x:c>
@@ -1186,8 +1303,10 @@
       <x:c r="J30" s="7" t="str">
         <x:v>Nhận diện theo số điện thoại; chờ PII policy.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="48" customHeight="1">
+      <x:c r="K30" s="7" t="str"/>
+      <x:c r="L30" s="7" t="str"/>
+    </x:row>
+    <x:row r="31" ht="50" customHeight="1">
       <x:c r="A31" s="7" t="str">
         <x:v>RW-002</x:v>
       </x:c>
@@ -1216,8 +1335,14 @@
       <x:c r="J31" s="7" t="str">
         <x:v>Mã thành viên là phương thức nhận diện riêng.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="48" customHeight="1">
+      <x:c r="K31" s="7" t="str">
+        <x:v>Chờ PO/BE nhận diện</x:v>
+      </x:c>
+      <x:c r="L31" s="7" t="str">
+        <x:v>BRD nêu phone/QR identification; mã thành viên riêng cần chốt định dạng, quyền và lookup trước khi thêm testcase.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="50" customHeight="1">
       <x:c r="A32" s="7" t="str">
         <x:v>RW-003</x:v>
       </x:c>
@@ -1248,8 +1373,14 @@
       <x:c r="J32" s="7" t="str">
         <x:v>Chưa có assertion khách bỏ qua Rewards nhưng vẫn thanh toán bình thường.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="48" customHeight="1">
+      <x:c r="K32" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L32" s="7" t="str">
+        <x:v>Bỏ qua Rewards/phone không cản trở đặt món và thanh toán; BR-QR-003. Payment contract còn chờ BE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="50" customHeight="1">
       <x:c r="A33" s="7" t="str">
         <x:v>RW-004</x:v>
       </x:c>
@@ -1280,8 +1411,10 @@
       <x:c r="J33" s="7" t="str">
         <x:v>Tra reward và eligibility theo rule PO.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="48" customHeight="1">
+      <x:c r="K33" s="7" t="str"/>
+      <x:c r="L33" s="7" t="str"/>
+    </x:row>
+    <x:row r="34" ht="50" customHeight="1">
       <x:c r="A34" s="7" t="str">
         <x:v>RW-005</x:v>
       </x:c>
@@ -1312,8 +1445,10 @@
       <x:c r="J34" s="7" t="str">
         <x:v>Áp reward hợp lệ vào bill chưa trả.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="48" customHeight="1">
+      <x:c r="K34" s="7" t="str"/>
+      <x:c r="L34" s="7" t="str"/>
+    </x:row>
+    <x:row r="35" ht="50" customHeight="1">
       <x:c r="A35" s="7" t="str">
         <x:v>RW-006</x:v>
       </x:c>
@@ -1344,8 +1479,14 @@
       <x:c r="J35" s="7" t="str">
         <x:v>P2 eligibility chung; cần riêng expired/used/insufficient points.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="48" customHeight="1">
+      <x:c r="K35" s="7" t="str">
+        <x:v>Chờ PO chốt rule</x:v>
+      </x:c>
+      <x:c r="L35" s="7" t="str">
+        <x:v>Tách expired, used và insufficient points thành ba bộ dữ liệu; hạn, balance, reason/code do PO/BE xác nhận.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="50" customHeight="1">
       <x:c r="A36" s="7" t="str">
         <x:v>RW-007</x:v>
       </x:c>
@@ -1374,8 +1515,14 @@
       <x:c r="J36" s="7" t="str">
         <x:v>Thiếu conflict stacking giữa các reward/promotion.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37" ht="48" customHeight="1">
+      <x:c r="K36" s="7" t="str">
+        <x:v>Chờ PO chốt rule</x:v>
+      </x:c>
+      <x:c r="L36" s="7" t="str">
+        <x:v>Chống cộng dồn reward/promotion cần ma trận cho phép/cấm và thứ tự áp dụng; chưa khẳng định mức giảm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="50" customHeight="1">
       <x:c r="A37" s="7" t="str">
         <x:v>RW-008</x:v>
       </x:c>
@@ -1404,8 +1551,14 @@
       <x:c r="J37" s="7" t="str">
         <x:v>Thiếu giới hạn khuyến mãi theo cấu hình/rule version.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="38" ht="48" customHeight="1">
+      <x:c r="K37" s="7" t="str">
+        <x:v>Chờ PO chốt rule</x:v>
+      </x:c>
+      <x:c r="L37" s="7" t="str">
+        <x:v>Giới hạn khuyến mãi, scope và rule version phải có cấu hình mẫu trước khi viết expected định lượng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="50" customHeight="1">
       <x:c r="A38" s="7" t="str">
         <x:v>RW-009</x:v>
       </x:c>
@@ -1434,8 +1587,14 @@
       <x:c r="J38" s="7" t="str">
         <x:v>Thiếu Supervisor override và audit.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="39" ht="48" customHeight="1">
+      <x:c r="K38" s="7" t="str">
+        <x:v>Chờ PO/BE quyền override</x:v>
+      </x:c>
+      <x:c r="L38" s="7" t="str">
+        <x:v>Chờ action, điều kiện Supervisor override, lý do, hiệu lực và audit schema; chưa suy ra endpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="50" customHeight="1">
       <x:c r="A39" s="7" t="str">
         <x:v>RW-010</x:v>
       </x:c>
@@ -1466,8 +1625,14 @@
       <x:c r="J39" s="7" t="str">
         <x:v>P2 double-use; retry cùng request key cần assertion ledger một lần.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="40" ht="48" customHeight="1">
+      <x:c r="K39" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L39" s="7" t="str">
+        <x:v>Retry cùng request key không tạo redemption/ledger trùng hoặc trừ điểm hai lần; key/status chờ BE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="50" customHeight="1">
       <x:c r="A40" s="7" t="str">
         <x:v>RW-011</x:v>
       </x:c>
@@ -1498,8 +1663,10 @@
       <x:c r="J40" s="7" t="str">
         <x:v>Concurrent redeem trên hai bill; balance không âm.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="41" ht="48" customHeight="1">
+      <x:c r="K40" s="7" t="str"/>
+      <x:c r="L40" s="7" t="str"/>
+    </x:row>
+    <x:row r="41" ht="50" customHeight="1">
       <x:c r="A41" s="7" t="str">
         <x:v>RW-012</x:v>
       </x:c>
@@ -1530,8 +1697,14 @@
       <x:c r="J41" s="7" t="str">
         <x:v>Payment failure có; CRM unavailable nhưng payment fallback cần case riêng.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42" ht="48" customHeight="1">
+      <x:c r="K41" s="7" t="str">
+        <x:v>Bổ sung assertion QA</x:v>
+      </x:c>
+      <x:c r="L41" s="7" t="str">
+        <x:v>CRM lỗi: có nhánh bỏ qua reward để tiếp tục thanh toán theo BRD risk note; cách fallback, role và ledger chờ PO/BE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="50" customHeight="1">
       <x:c r="A42" s="7" t="str">
         <x:v>RW-013</x:v>
       </x:c>
@@ -1560,10 +1733,12 @@
         <x:v>Khớp</x:v>
       </x:c>
       <x:c r="J42" s="7" t="str">
-        <x:v>≤30 giây tạm theo mục tiêu; PO cần chốt với risk note ≤10 giây.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="48" customHeight="1">
+        <x:v>BRD nêu Rewards ≤30s ở mục tiêu, ≤10s ở risk note và ≤3s ở bảng target; PO chốt mốc/điểm đo trước khi test.</x:v>
+      </x:c>
+      <x:c r="K42" s="7" t="str"/>
+      <x:c r="L42" s="7" t="str"/>
+    </x:row>
+    <x:row r="43" ht="50" customHeight="1">
       <x:c r="A43" s="7" t="str">
         <x:v>RW-014</x:v>
       </x:c>
@@ -1594,8 +1769,10 @@
       <x:c r="J43" s="7" t="str">
         <x:v>Gỡ reward trước pay và hoàn nguyên ledger.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44" ht="48" customHeight="1">
+      <x:c r="K43" s="7" t="str"/>
+      <x:c r="L43" s="7" t="str"/>
+    </x:row>
+    <x:row r="44" ht="50" customHeight="1">
       <x:c r="A44" s="7" t="str">
         <x:v>RW-015</x:v>
       </x:c>
@@ -1626,8 +1803,10 @@
       <x:c r="J44" s="7" t="str">
         <x:v>Không lộ PII/points cross-customer/outlet.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="48" customHeight="1">
+      <x:c r="K44" s="7" t="str"/>
+      <x:c r="L44" s="7" t="str"/>
+    </x:row>
+    <x:row r="45" ht="50" customHeight="1">
       <x:c r="A45" s="7" t="str">
         <x:v>RW-016</x:v>
       </x:c>
@@ -1658,8 +1837,14 @@
       <x:c r="J45" s="7" t="str">
         <x:v>P2 payment failed; refund/hủy sau pay và reversal thiếu.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="46" ht="48" customHeight="1">
+      <x:c r="K45" s="7" t="str">
+        <x:v>Chờ PO chốt reversal</x:v>
+      </x:c>
+      <x:c r="L45" s="7" t="str">
+        <x:v>Phân biệt payment failed, hủy và refund sau PAID; thời điểm/amount hoàn điểm cần PO/Finance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="50" customHeight="1">
       <x:c r="A46" s="7" t="str">
         <x:v>RW-017</x:v>
       </x:c>
@@ -1690,8 +1875,14 @@
       <x:c r="J46" s="7" t="str">
         <x:v>Eligibility lần đầu có; thay bill rồi tính lại chưa có.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47" ht="48" customHeight="1">
+      <x:c r="K46" s="7" t="str">
+        <x:v>Chờ PO chốt rule</x:v>
+      </x:c>
+      <x:c r="L46" s="7" t="str">
+        <x:v>Bill đổi thì tái đánh giá eligibility là draft; chốt điều kiện và thời điểm tính lại.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="50" customHeight="1">
       <x:c r="A47" s="7" t="str">
         <x:v>RW-018</x:v>
       </x:c>
@@ -1722,8 +1913,10 @@
       <x:c r="J47" s="7" t="str">
         <x:v>Earn đúng một lần sau PAID.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48" ht="48" customHeight="1">
+      <x:c r="K47" s="7" t="str"/>
+      <x:c r="L47" s="7" t="str"/>
+    </x:row>
+    <x:row r="48" ht="50" customHeight="1">
       <x:c r="A48" s="7" t="str">
         <x:v>RW-019</x:v>
       </x:c>
@@ -1754,8 +1947,14 @@
       <x:c r="J48" s="7" t="str">
         <x:v>Earn/balance có; thiếu ledger redemption/reversal đầy đủ.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49" ht="48" customHeight="1">
+      <x:c r="K48" s="7" t="str">
+        <x:v>Chờ PO/BE ledger</x:v>
+      </x:c>
+      <x:c r="L48" s="7" t="str">
+        <x:v>Tách earn, redeem, reversal trong history; field, trạng thái và đối soát chờ contract/Finance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="50" customHeight="1">
       <x:c r="A49" s="7" t="str">
         <x:v>RW-020</x:v>
       </x:c>
@@ -1785,6 +1984,12 @@
       </x:c>
       <x:c r="J49" s="7" t="str">
         <x:v>P2 apply reward có; thiếu giả mạo discount từ client.</x:v>
+      </x:c>
+      <x:c r="K49" s="7" t="str">
+        <x:v>Chờ PO/BE giá trị giảm</x:v>
+      </x:c>
+      <x:c r="L49" s="7" t="str">
+        <x:v>Không tin discount từ client; xác định reject hay bỏ qua field, mã lỗi và giá tính server sau contract.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -1857,10 +2062,61 @@
       <x:c r="I56" s="15"/>
       <x:c r="J56" s="15"/>
     </x:row>
+    <x:row r="58" ht="42" customHeight="1">
+      <x:c r="A58" t="str">
+        <x:v>P2-only cần nối scope</x:v>
+      </x:c>
+      <x:c r="B58" s="15" t="str">
+        <x:v>P2-QR-010: giá giả mạo (case bảo mật riêng); P2-RWD-002: SĐT trùng (nhánh RW-001); P2-RWD-008: sửa sau PAID (nhánh RW-014). Không gắn ép vào case khác mục tiêu.</x:v>
+      </x:c>
+      <x:c r="C58" s="15"/>
+      <x:c r="D58" s="15"/>
+      <x:c r="E58" s="15"/>
+      <x:c r="F58" s="15"/>
+      <x:c r="G58" s="15"/>
+      <x:c r="H58" s="15"/>
+      <x:c r="I58" s="15"/>
+      <x:c r="J58" s="15"/>
+    </x:row>
+    <x:row r="59" ht="42" customHeight="1">
+      <x:c r="A59" t="str">
+        <x:v>Quy tắc PO cần chốt</x:v>
+      </x:c>
+      <x:c r="B59" s="15" t="str">
+        <x:v>Rewards SLA trong BRD: ≤30s, ≤10s, ≤3s; quyền Customer apply reward ở các bảng vai trò chưa thống nhất. Giữ expected định lượng/quyền ở TBD.</x:v>
+      </x:c>
+      <x:c r="C59" s="15"/>
+      <x:c r="D59" s="15"/>
+      <x:c r="E59" s="15"/>
+      <x:c r="F59" s="15"/>
+      <x:c r="G59" s="15"/>
+      <x:c r="H59" s="15"/>
+      <x:c r="I59" s="15"/>
+      <x:c r="J59" s="15"/>
+    </x:row>
+    <x:row r="60" ht="42" customHeight="1">
+      <x:c r="A60" t="str">
+        <x:v>Gate thực thi</x:v>
+      </x:c>
+      <x:c r="B60" s="15" t="str">
+        <x:v>ENV-QA-04 chờ BE; không có endpoint/fixture QR/Rewards trên staging 46d6049. 44 case vẫn Not Executed.</x:v>
+      </x:c>
+      <x:c r="C60" s="15"/>
+      <x:c r="D60" s="15"/>
+      <x:c r="E60" s="15"/>
+      <x:c r="F60" s="15"/>
+      <x:c r="G60" s="15"/>
+      <x:c r="H60" s="15"/>
+      <x:c r="I60" s="15"/>
+      <x:c r="J60" s="15"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="B55:J55"/>
     <x:mergeCell ref="B56:J56"/>
+    <x:mergeCell ref="B58:J58"/>
+    <x:mergeCell ref="B59:J59"/>
+    <x:mergeCell ref="B60:J60"/>
   </x:mergeCells>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G6:G49">

</xml_diff>

<commit_message>
qa: link rewards duplicate identity and document P2-only cases
</commit_message>
<xml_diff>
--- a/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
+++ b/qa/automation/Testing_POS/planning/PLN_QA_03_QR_RW_Trace_2026-10-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R108336a74ceb42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R8290e56d2b724076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace QR Rewards" sheetId="1" r:id="R21399a71dedf4845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="2" r:id="R887e3aa196844c20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1295,13 +1295,13 @@
         <x:v>Not Executed</x:v>
       </x:c>
       <x:c r="H30" s="7" t="str">
-        <x:v>P2-RWD-001</x:v>
+        <x:v>P2-RWD-001; P2-RWD-002</x:v>
       </x:c>
       <x:c r="I30" s="7" t="str">
         <x:v>Khớp</x:v>
       </x:c>
       <x:c r="J30" s="7" t="str">
-        <x:v>Nhận diện theo số điện thoại; chờ PII policy.</x:v>
+        <x:v>Nhận diện SĐT: lookup/profile và nhánh trùng SĐT không tạo hai profile; P2-RWD-002 là kiểm tra idempotency liên quan.</x:v>
       </x:c>
       <x:c r="K30" s="7" t="str"/>
       <x:c r="L30" s="7" t="str"/>
@@ -2035,7 +2035,7 @@
         <x:v>P2 QR/RWD chưa có Sprint 3 ID trực tiếp</x:v>
       </x:c>
       <x:c r="B55" s="15" t="str">
-        <x:v>P2-QR-010; P2-RWD-002; P2-RWD-008</x:v>
+        <x:v>P2-QR-010; P2-RWD-008</x:v>
       </x:c>
       <x:c r="C55" s="15"/>
       <x:c r="D55" s="15"/>
@@ -2067,7 +2067,7 @@
         <x:v>P2-only cần nối scope</x:v>
       </x:c>
       <x:c r="B58" s="15" t="str">
-        <x:v>P2-QR-010: giá giả mạo (case bảo mật riêng); P2-RWD-002: SĐT trùng (nhánh RW-001); P2-RWD-008: sửa sau PAID (nhánh RW-014). Không gắn ép vào case khác mục tiêu.</x:v>
+        <x:v>P2-RWD-002 nối RW-001 (trùng SĐT). P2-QR-010 kiểm giá client giả mạo và P2-RWD-008 chặn sửa sau PAID vẫn là P2-only; đề xuất ID Sprint 3 mới chỉ sau khi duyệt scope.</x:v>
       </x:c>
       <x:c r="C58" s="15"/>
       <x:c r="D58" s="15"/>
@@ -2083,7 +2083,7 @@
         <x:v>Quy tắc PO cần chốt</x:v>
       </x:c>
       <x:c r="B59" s="15" t="str">
-        <x:v>Rewards SLA trong BRD: ≤30s, ≤10s, ≤3s; quyền Customer apply reward ở các bảng vai trò chưa thống nhất. Giữ expected định lượng/quyền ở TBD.</x:v>
+        <x:v>PO chốt SLA Rewards (BRD nêu ≤30s, ≤10s và ≤3s), quyền Customer apply reward và chính sách case P2-only trước khi định lượng Expected Result.</x:v>
       </x:c>
       <x:c r="C59" s="15"/>
       <x:c r="D59" s="15"/>

</xml_diff>